<commit_message>
correct rule category diastolic and hr
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-DSE.xlsx
+++ b/baseline/data_processing_elements-DSE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Documents\Boulot\ProPASS\DPE_V2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9FD2AD8-591E-4238-97AE-8549E610F6D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E89451C-F1BC-4B83-BB00-DFDC6373EDA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4660,7 +4660,7 @@
         <v>50</v>
       </c>
       <c r="Y37" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="Z37" s="8" t="s">
         <v>651</v>
@@ -4722,7 +4722,7 @@
         <v>50</v>
       </c>
       <c r="Y38" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="Z38" s="8" t="s">
         <v>652</v>

</xml_diff>